<commit_message>
own group matches and player db conflict
</commit_message>
<xml_diff>
--- a/samples_csv/sing.xlsx
+++ b/samples_csv/sing.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Relative\Projects\seva projects\badminton\society-badminton-app\samples_csv\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3C97E1C-4DD7-4D31-B230-5278D225BF85}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EA357B37-B9C5-489C-9F68-5ACA5D08A2A2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2846" yWindow="2846" windowWidth="18514" windowHeight="10740" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="12257" yWindow="0" windowWidth="12514" windowHeight="14794" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="98" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="50">
   <si>
     <t>MHT Id</t>
   </si>
@@ -174,13 +174,7 @@
     <t>Abhist Pal</t>
   </si>
   <si>
-    <t>Badminton Singles</t>
-  </si>
-  <si>
     <t>Mobile</t>
-  </si>
-  <si>
-    <t>badminton_singles</t>
   </si>
 </sst>
 </file>
@@ -529,13 +523,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D48"/>
+  <dimension ref="A1:C48"/>
   <sheetFormatPr defaultRowHeight="14.6" x14ac:dyDescent="0.4"/>
   <cols>
-    <col min="4" max="4" width="10.84375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.15234375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.84375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -545,665 +540,521 @@
       <c r="C1" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.4">
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A2" s="2">
         <v>119420</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D2" s="2">
+      <c r="C2" s="2">
         <v>8469091699</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A3" s="2">
         <v>126888</v>
       </c>
       <c r="B3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="C3" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D3" s="2">
+      <c r="C3" s="2">
         <v>8879939998</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A4" s="2">
         <v>129694</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="C4" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D4" s="2">
+      <c r="C4" s="2">
         <v>9426242325</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A5" s="2">
         <v>133348</v>
       </c>
       <c r="B5" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="C5" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D5" s="2">
+      <c r="C5" s="2">
         <v>9016255414</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A6" s="2">
         <v>135304</v>
       </c>
       <c r="B6" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D6" s="2">
+      <c r="C6" s="2">
         <v>9638565431</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A7" s="2">
         <v>135596</v>
       </c>
       <c r="B7" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="C7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D7" s="2">
+      <c r="C7" s="2">
         <v>9924629232</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A8" s="2">
         <v>138340</v>
       </c>
       <c r="B8" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="C8" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D8" s="2">
+      <c r="C8" s="2">
         <v>7046894277</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A9" s="2">
         <v>143412</v>
       </c>
       <c r="B9" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D9" s="2">
+      <c r="C9" s="2">
         <v>7405811791</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A10" s="2">
         <v>144635</v>
       </c>
       <c r="B10" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D10" s="2">
+      <c r="C10" s="2">
         <v>8087700757</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A11" s="2">
         <v>146170</v>
       </c>
       <c r="B11" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C11" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D11" s="2">
+      <c r="C11" s="2">
         <v>6353232254</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A12" s="2">
         <v>150538</v>
       </c>
       <c r="B12" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="C12" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D12" s="2">
+      <c r="C12" s="2">
         <v>9171213176</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A13" s="2">
         <v>151148</v>
       </c>
       <c r="B13" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D13" s="2">
+      <c r="C13" s="2">
         <v>9552612512</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A14" s="2">
         <v>151693</v>
       </c>
       <c r="B14" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="C14" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D14" s="2">
+      <c r="C14" s="2">
         <v>7096493425</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A15" s="2">
         <v>151918</v>
       </c>
       <c r="B15" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C15" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D15" s="2">
+      <c r="C15" s="2">
         <v>9316630864</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A16" s="2">
         <v>152061</v>
       </c>
       <c r="B16" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="C16" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D16" s="2">
+      <c r="C16" s="2">
         <v>9426923974</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A17" s="2">
         <v>153864</v>
       </c>
       <c r="B17" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="C17" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D17" s="2">
+      <c r="C17" s="2">
         <v>8303003968</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A18" s="2">
         <v>153870</v>
       </c>
       <c r="B18" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C18" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D18" s="2">
+      <c r="C18" s="2">
         <v>9409523384</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A19" s="2">
         <v>154481</v>
       </c>
       <c r="B19" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="C19" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D19" s="2">
+      <c r="C19" s="2">
         <v>9926910037</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A20" s="2">
         <v>156591</v>
       </c>
       <c r="B20" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="C20" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D20" s="2">
+      <c r="C20" s="2">
         <v>7387166531</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A21" s="2">
         <v>157346</v>
       </c>
       <c r="B21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="C21" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D21" s="2">
+      <c r="C21" s="2">
         <v>7434849356</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A22" s="2">
         <v>157717</v>
       </c>
       <c r="B22" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="C22" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D22" s="2">
+      <c r="C22" s="2">
         <v>9500057221</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A23" s="2">
         <v>161741</v>
       </c>
       <c r="B23" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="C23" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D23" s="2">
+      <c r="C23" s="2">
         <v>7016818654</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A24" s="2">
         <v>165099</v>
       </c>
       <c r="B24" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="C24" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D24" s="2">
+      <c r="C24" s="2">
         <v>9664642952</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A25" s="2">
         <v>168607</v>
       </c>
       <c r="B25" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="C25" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D25" s="2">
+      <c r="C25" s="2">
         <v>9256756142</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A26" s="2">
         <v>27755</v>
       </c>
       <c r="B26" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C26" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D26" s="2">
+      <c r="C26" s="2">
         <v>9429601783</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A27" s="2">
         <v>34064</v>
       </c>
       <c r="B27" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C27" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D27" s="2">
+      <c r="C27" s="2">
         <v>8980772697</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A28" s="2">
         <v>34744</v>
       </c>
       <c r="B28" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="C28" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D28" s="2">
+      <c r="C28" s="2">
         <v>9924343846</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A29" s="2">
         <v>60460</v>
       </c>
       <c r="B29" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="C29" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D29" s="2">
+      <c r="C29" s="2">
         <v>8866765593</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A30" s="2">
         <v>64311</v>
       </c>
       <c r="B30" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="C30" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D30" s="2">
+      <c r="C30" s="2">
         <v>8866833278</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A31" s="2">
         <v>68329</v>
       </c>
       <c r="B31" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="C31" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D31" s="2">
+      <c r="C31" s="2">
         <v>7984532152</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A32" s="2">
         <v>90132</v>
       </c>
       <c r="B32" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="C32" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D32" s="2">
+      <c r="C32" s="2">
         <v>7984499214</v>
       </c>
     </row>
-    <row r="33" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A33" s="2">
         <v>93658</v>
       </c>
       <c r="B33" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="C33" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D33" s="2">
+      <c r="C33" s="2">
         <v>7283980302</v>
       </c>
     </row>
-    <row r="34" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A34" s="2">
         <v>124192</v>
       </c>
       <c r="B34" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="C34" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D34" s="2">
+      <c r="C34" s="2">
         <v>8200544566</v>
       </c>
     </row>
-    <row r="35" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A35" s="2">
         <v>138990</v>
       </c>
       <c r="B35" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C35" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D35" s="2">
+      <c r="C35" s="2">
         <v>7359366133</v>
       </c>
     </row>
-    <row r="36" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A36" s="2">
         <v>140179</v>
       </c>
       <c r="B36" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C36" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D36" s="2">
+      <c r="C36" s="2">
         <v>8160847528</v>
       </c>
     </row>
-    <row r="37" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A37" s="2">
         <v>140180</v>
       </c>
       <c r="B37" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C37" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D37" s="2">
+      <c r="C37" s="2">
         <v>8347806960</v>
       </c>
     </row>
-    <row r="38" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A38" s="2">
         <v>140952</v>
       </c>
       <c r="B38" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="C38" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D38" s="2">
+      <c r="C38" s="2">
         <v>7877057956</v>
       </c>
     </row>
-    <row r="39" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A39" s="2">
         <v>142768</v>
       </c>
       <c r="B39" s="2" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D39" s="2">
+      <c r="C39" s="2">
         <v>9723033052</v>
       </c>
     </row>
-    <row r="40" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A40" s="2">
         <v>144184</v>
       </c>
       <c r="B40" s="2" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D40" s="2">
+      <c r="C40" s="2">
         <v>7077902158</v>
       </c>
     </row>
-    <row r="41" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A41" s="2">
         <v>154716</v>
       </c>
       <c r="B41" s="2" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D41" s="2">
+      <c r="C41" s="2">
         <v>8401522921</v>
       </c>
     </row>
-    <row r="42" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A42" s="2">
         <v>155511</v>
       </c>
       <c r="B42" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D42" s="2">
+      <c r="C42" s="2">
         <v>9428175629</v>
       </c>
     </row>
-    <row r="43" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A43" s="2">
         <v>3850</v>
       </c>
       <c r="B43" s="2" t="s">
         <v>43</v>
       </c>
-      <c r="C43" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D43" s="2">
+      <c r="C43" s="2">
         <v>9574004343</v>
       </c>
     </row>
-    <row r="44" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A44" s="2">
         <v>39352</v>
       </c>
       <c r="B44" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C44" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D44" s="2">
+      <c r="C44" s="2">
         <v>9924343811</v>
       </c>
     </row>
-    <row r="45" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A45" s="2">
         <v>48737</v>
       </c>
       <c r="B45" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="C45" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D45" s="2">
+      <c r="C45" s="2">
         <v>9924884777</v>
       </c>
     </row>
-    <row r="46" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A46" s="2">
         <v>65407</v>
       </c>
       <c r="B46" s="2" t="s">
         <v>46</v>
       </c>
-      <c r="C46" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D46" s="2">
+      <c r="C46" s="2">
         <v>7698275609</v>
       </c>
     </row>
-    <row r="47" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A47" s="2">
         <v>85171</v>
       </c>
       <c r="B47" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="C47" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D47" s="2">
+      <c r="C47" s="2">
         <v>9601429647</v>
       </c>
     </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.4">
       <c r="A48" s="2">
         <v>85471</v>
       </c>
       <c r="B48" s="2" t="s">
         <v>48</v>
       </c>
-      <c r="C48" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="D48" s="2">
+      <c r="C48" s="2">
         <v>9406560055</v>
       </c>
     </row>

</xml_diff>